<commit_message>
Add Wikidata IRIs to resources (#98)
</commit_message>
<xml_diff>
--- a/data/daschland_ontology/daschland (Alice in DaSCHland)/properties.xlsx
+++ b/data/daschland_ontology/daschland (Alice in DaSCHland)/properties.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noemivillars-amberg/Documents/daschland-scripts/data/daschland_ontology/daschland (Alice in DaSCHland)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noraammann/Documents/Cloned_GitHub/daschland-scripts/data/daschland_ontology/daschland (Alice in DaSCHland)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1687B0D2-B308-0A44-907D-669F1923C0BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B4E33A-4112-3D44-AD04-AB17E77BC38C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3800" yWindow="620" windowWidth="68740" windowHeight="30240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Q$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Q$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -173,7 +173,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="361">
   <si>
     <t>name</t>
   </si>
@@ -1238,18 +1238,50 @@
   </si>
   <si>
     <t>:StoryChapter</t>
+  </si>
+  <si>
+    <t>Wikidata ID</t>
+  </si>
+  <si>
+    <t>link to the corresponding Wikidata entry</t>
+  </si>
+  <si>
+    <t>link zu der Wikidata Seite</t>
+  </si>
+  <si>
+    <t>lien vers l'entrée Wikidata correspondante</t>
+  </si>
+  <si>
+    <t>link alla voce Wikidata corrispondente</t>
+  </si>
+  <si>
+    <t>hasWikidataLink</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1357,7 +1389,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1367,6 +1399,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79995117038483843"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1383,25 +1421,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2230,7 +2270,7 @@
       <c r="J15" t="s">
         <v>316</v>
       </c>
-      <c r="L15" s="4" t="s">
+      <c r="L15" s="18" t="s">
         <v>110</v>
       </c>
       <c r="M15" s="4" t="s">
@@ -2515,7 +2555,7 @@
       <c r="J22" t="s">
         <v>322</v>
       </c>
-      <c r="L22" s="4" t="s">
+      <c r="L22" s="18" t="s">
         <v>153</v>
       </c>
       <c r="M22" s="4" t="s">
@@ -2526,116 +2566,114 @@
       </c>
     </row>
     <row r="23" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="C23" t="s">
-        <v>157</v>
-      </c>
-      <c r="D23" t="s">
-        <v>158</v>
-      </c>
-      <c r="E23" t="s">
-        <v>159</v>
-      </c>
-      <c r="G23" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="H23" t="s">
-        <v>295</v>
-      </c>
-      <c r="I23" t="s">
-        <v>239</v>
-      </c>
-      <c r="J23" t="s">
-        <v>323</v>
-      </c>
-      <c r="L23" s="4" t="s">
-        <v>160</v>
+      <c r="A23" s="19" t="s">
+        <v>360</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="D23" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="G23" s="18" t="s">
+        <v>356</v>
+      </c>
+      <c r="H23" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="I23" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="J23" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="L23" s="18" t="s">
+        <v>110</v>
       </c>
       <c r="M23" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="N23" s="4" t="s">
-        <v>162</v>
+        <v>154</v>
+      </c>
+      <c r="N23" s="18" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="16" t="s">
-        <v>353</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>346</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>345</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>344</v>
-      </c>
-      <c r="E24" s="15" t="s">
-        <v>347</v>
-      </c>
-      <c r="G24" s="15" t="s">
-        <v>348</v>
-      </c>
-      <c r="H24" s="15" t="s">
-        <v>349</v>
-      </c>
-      <c r="I24" s="15" t="s">
-        <v>350</v>
-      </c>
-      <c r="J24" s="15" t="s">
-        <v>351</v>
+      <c r="A24" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C24" t="s">
+        <v>157</v>
+      </c>
+      <c r="D24" t="s">
+        <v>158</v>
+      </c>
+      <c r="E24" t="s">
+        <v>159</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="H24" t="s">
+        <v>295</v>
+      </c>
+      <c r="I24" t="s">
+        <v>239</v>
+      </c>
+      <c r="J24" t="s">
+        <v>323</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="M24" s="17" t="s">
-        <v>354</v>
+        <v>160</v>
+      </c>
+      <c r="M24" s="4" t="s">
+        <v>161</v>
       </c>
       <c r="N24" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="P24" s="4"/>
-      <c r="Q24" s="4"/>
+        <v>162</v>
+      </c>
     </row>
     <row r="25" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="12" t="s">
-        <v>338</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>339</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>342</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>340</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="G25" s="13" t="s">
-        <v>339</v>
-      </c>
-      <c r="H25" s="13" t="s">
-        <v>342</v>
-      </c>
-      <c r="I25" s="13" t="s">
-        <v>340</v>
-      </c>
-      <c r="J25" s="4" t="s">
-        <v>341</v>
+      <c r="A25" s="16" t="s">
+        <v>353</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>346</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>345</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>344</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>347</v>
+      </c>
+      <c r="G25" s="15" t="s">
+        <v>348</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>349</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>350</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>351</v>
       </c>
       <c r="L25" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="M25" s="13" t="s">
-        <v>178</v>
+      <c r="M25" s="17" t="s">
+        <v>354</v>
       </c>
       <c r="N25" s="4" t="s">
         <v>164</v>
@@ -2644,38 +2682,38 @@
       <c r="Q25" s="4"/>
     </row>
     <row r="26" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="D26" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="E26" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>274</v>
-      </c>
-      <c r="H26" t="s">
-        <v>296</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>276</v>
-      </c>
-      <c r="J26" t="s">
-        <v>324</v>
+      <c r="A26" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>342</v>
+      </c>
+      <c r="I26" s="13" t="s">
+        <v>340</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>341</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="M26" s="4" t="s">
-        <v>167</v>
+        <v>163</v>
+      </c>
+      <c r="M26" s="13" t="s">
+        <v>178</v>
       </c>
       <c r="N26" s="4" t="s">
         <v>164</v>
@@ -2684,76 +2722,78 @@
       <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="16" t="s">
-        <v>352</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C27" t="s">
-        <v>169</v>
-      </c>
-      <c r="D27" t="s">
-        <v>170</v>
-      </c>
-      <c r="E27" t="s">
-        <v>171</v>
+      <c r="A27" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>256</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="H27" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J27" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="M27" s="17" t="s">
-        <v>354</v>
+        <v>166</v>
+      </c>
+      <c r="M27" s="4" t="s">
+        <v>167</v>
       </c>
       <c r="N27" s="4" t="s">
         <v>164</v>
       </c>
+      <c r="P27" s="4"/>
+      <c r="Q27" s="4"/>
     </row>
     <row r="28" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="D28" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="E28" s="8" t="s">
-        <v>269</v>
+      <c r="A28" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C28" t="s">
+        <v>169</v>
+      </c>
+      <c r="D28" t="s">
+        <v>170</v>
+      </c>
+      <c r="E28" t="s">
+        <v>171</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>214</v>
+        <v>251</v>
       </c>
       <c r="H28" t="s">
-        <v>298</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>240</v>
+        <v>297</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>275</v>
       </c>
       <c r="J28" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="M28" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
+      </c>
+      <c r="M28" s="17" t="s">
+        <v>354</v>
       </c>
       <c r="N28" s="4" t="s">
         <v>164</v>
@@ -2761,71 +2801,69 @@
     </row>
     <row r="29" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="H29" s="4" t="s">
-        <v>299</v>
+        <v>214</v>
+      </c>
+      <c r="H29" t="s">
+        <v>298</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="J29" s="4" t="s">
-        <v>327</v>
+        <v>240</v>
+      </c>
+      <c r="J29" t="s">
+        <v>326</v>
       </c>
       <c r="L29" s="4" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="N29" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="P29" s="4"/>
-      <c r="Q29" s="4"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="C30" t="s">
-        <v>181</v>
+        <v>176</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>258</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E30" t="s">
-        <v>183</v>
+        <v>262</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>273</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>221</v>
-      </c>
-      <c r="H30" t="s">
-        <v>300</v>
-      </c>
-      <c r="I30" t="s">
-        <v>242</v>
-      </c>
-      <c r="J30" t="s">
-        <v>328</v>
+        <v>215</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>327</v>
       </c>
       <c r="L30" s="4" t="s">
         <v>177</v>
@@ -2836,34 +2874,36 @@
       <c r="N30" s="4" t="s">
         <v>164</v>
       </c>
+      <c r="P30" s="4"/>
+      <c r="Q30" s="4"/>
     </row>
     <row r="31" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="C31" t="s">
-        <v>186</v>
-      </c>
-      <c r="D31" t="s">
-        <v>187</v>
+        <v>181</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>182</v>
       </c>
       <c r="E31" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H31" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I31" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J31" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="L31" s="4" t="s">
         <v>177</v>
@@ -2877,37 +2917,37 @@
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>264</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>259</v>
-      </c>
-      <c r="D32" s="8" t="s">
-        <v>263</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>270</v>
+        <v>184</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C32" t="s">
+        <v>186</v>
+      </c>
+      <c r="D32" t="s">
+        <v>187</v>
+      </c>
+      <c r="E32" t="s">
+        <v>188</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="H32" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I32" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="J32" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L32" s="4" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="M32" s="4" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="N32" s="4" t="s">
         <v>164</v>
@@ -2915,37 +2955,37 @@
     </row>
     <row r="33" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="H33" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="I33" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="J33" s="4" t="s">
-        <v>331</v>
+        <v>216</v>
+      </c>
+      <c r="H33" t="s">
+        <v>302</v>
+      </c>
+      <c r="I33" t="s">
+        <v>244</v>
+      </c>
+      <c r="J33" t="s">
+        <v>330</v>
       </c>
       <c r="L33" s="4" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="M33" s="4" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="N33" s="4" t="s">
         <v>164</v>
@@ -2953,122 +2993,159 @@
     </row>
     <row r="34" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="C34" t="s">
-        <v>197</v>
-      </c>
-      <c r="D34" t="s">
-        <v>198</v>
-      </c>
-      <c r="E34" t="s">
-        <v>199</v>
+        <v>265</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>266</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>271</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="H34" t="s">
-        <v>304</v>
-      </c>
-      <c r="I34" t="s">
-        <v>246</v>
-      </c>
-      <c r="J34" t="s">
-        <v>332</v>
+        <v>217</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="J34" s="4" t="s">
+        <v>331</v>
       </c>
       <c r="L34" s="4" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="M34" s="4" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="N34" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="P34" s="4"/>
     </row>
     <row r="35" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>267</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>254</v>
+        <v>196</v>
+      </c>
+      <c r="C35" t="s">
+        <v>197</v>
+      </c>
+      <c r="D35" t="s">
+        <v>198</v>
+      </c>
+      <c r="E35" t="s">
+        <v>199</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H35" t="s">
-        <v>305</v>
-      </c>
-      <c r="I35" s="4" t="s">
-        <v>247</v>
+        <v>304</v>
+      </c>
+      <c r="I35" t="s">
+        <v>246</v>
       </c>
       <c r="J35" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="L35" s="4" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="M35" s="4" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="N35" s="4" t="s">
         <v>164</v>
       </c>
       <c r="P35" s="4"/>
-      <c r="Q35" s="4"/>
     </row>
     <row r="36" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H36" t="s">
-        <v>306</v>
-      </c>
-      <c r="I36" t="s">
-        <v>248</v>
+        <v>305</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>247</v>
       </c>
       <c r="J36" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="L36" s="4" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="M36" s="4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="N36" s="4" t="s">
         <v>164</v>
       </c>
+      <c r="P36" s="4"/>
+      <c r="Q36" s="4"/>
     </row>
-    <row r="37" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="37" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>268</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="G37" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="H37" t="s">
+        <v>306</v>
+      </c>
+      <c r="I37" t="s">
+        <v>248</v>
+      </c>
+      <c r="J37" t="s">
+        <v>334</v>
+      </c>
+      <c r="L37" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="M37" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="N37" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
     <row r="38" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="39" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="40" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3945,7 +4022,7 @@
     <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <autoFilter ref="A1:Q36" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:Q37" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="A1" r:id="rId1" location="property-name" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B1" r:id="rId2" location="property-labels" xr:uid="{00000000-0004-0000-0000-000001000000}"/>

</xml_diff>

<commit_message>
feat: add data-license and -copyright owner to the JSON (#122)
</commit_message>
<xml_diff>
--- a/data/daschland_ontology/daschland (Alice in DaSCHland)/properties.xlsx
+++ b/data/daschland_ontology/daschland (Alice in DaSCHland)/properties.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noraammann/Documents/Cloned_GitHub/daschland-scripts/data/daschland_ontology/daschland (Alice in DaSCHland)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/noraammann/Documents/Cloned_GitHub/0854-daschland-scripts/data/daschland_ontology/daschland (Alice in DaSCHland)/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B4E33A-4112-3D44-AD04-AB17E77BC38C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F33C0C-530C-9B47-940F-D9B38638A2A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="20460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Q$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Q$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -173,7 +173,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="350">
   <si>
     <t>name</t>
   </si>
@@ -532,30 +532,6 @@
     <t>hlist: Keyword</t>
   </si>
   <si>
-    <t>hasLicenseList</t>
-  </si>
-  <si>
-    <t>License</t>
-  </si>
-  <si>
-    <t>Lizenz</t>
-  </si>
-  <si>
-    <t>Licence</t>
-  </si>
-  <si>
-    <t>Licenza</t>
-  </si>
-  <si>
-    <t>License of use of the Media file</t>
-  </si>
-  <si>
-    <t>hasValue, schema:license</t>
-  </si>
-  <si>
-    <t>hlist: License</t>
-  </si>
-  <si>
     <t>hasName</t>
   </si>
   <si>
@@ -877,9 +853,6 @@
     <t>Identifiant unique</t>
   </si>
   <si>
-    <t>Licence d'utilisation du fichier média</t>
-  </si>
-  <si>
     <t>Citation, telle qu'elle est écrite dans l'histoire originale</t>
   </si>
   <si>
@@ -1045,9 +1018,6 @@
     <t>Mit dem Datensatz verbundene Schlüsselwörter</t>
   </si>
   <si>
-    <t>Lizenz zur Nutzung der Mediendatei</t>
-  </si>
-  <si>
     <t>Zitat, wie im Originaltext geschrieben</t>
   </si>
   <si>
@@ -1127,9 +1097,6 @@
   </si>
   <si>
     <t>Parole chiave associate alla scheda</t>
-  </si>
-  <si>
-    <t>Licenza d'uso del file multimediale</t>
   </si>
   <si>
     <t>Citazione, come riportata nella storia originale</t>
@@ -1657,7 +1624,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q912"/>
+  <dimension ref="A1:Q911"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27.33203125" customWidth="1"/>
@@ -1727,21 +1694,21 @@
         <v>14</v>
       </c>
       <c r="P1" s="10" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="E2" s="4" t="s">
         <v>15</v>
@@ -1750,13 +1717,13 @@
         <v>16</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="L2" s="4" t="s">
         <v>17</v>
@@ -1788,13 +1755,13 @@
         <v>25</v>
       </c>
       <c r="H3" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="I3" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="J3" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="L3" s="4" t="s">
         <v>26</v>
@@ -1803,7 +1770,7 @@
         <v>18</v>
       </c>
       <c r="N3" s="14" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -1826,10 +1793,10 @@
         <v>33</v>
       </c>
       <c r="H4" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="I4" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="J4" t="s">
         <v>32</v>
@@ -1905,13 +1872,13 @@
         <v>48</v>
       </c>
       <c r="H6" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="I6" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="J6" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="L6" s="4" t="s">
         <v>49</v>
@@ -1945,7 +1912,7 @@
         <v>55</v>
       </c>
       <c r="H7" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="I7" t="s">
         <v>53</v>
@@ -1987,7 +1954,7 @@
         <v>61</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="J8" s="4" t="s">
         <v>62</v>
@@ -2024,13 +1991,13 @@
         <v>69</v>
       </c>
       <c r="H9" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="L9" s="4" t="s">
         <v>63</v>
@@ -2042,7 +2009,7 @@
         <v>27</v>
       </c>
       <c r="P9" s="11" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="Q9" s="4"/>
     </row>
@@ -2066,13 +2033,13 @@
         <v>75</v>
       </c>
       <c r="H10" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="J10" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="L10" s="4" t="s">
         <v>76</v>
@@ -2107,13 +2074,13 @@
         <v>85</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="J11" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
       <c r="L11" s="4" t="s">
         <v>86</v>
@@ -2146,13 +2113,13 @@
         <v>92</v>
       </c>
       <c r="H12" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="I12" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="J12" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="L12" s="4" t="s">
         <v>93</v>
@@ -2184,13 +2151,13 @@
         <v>96</v>
       </c>
       <c r="H13" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="J13" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="L13" s="4" t="s">
         <v>97</v>
@@ -2224,13 +2191,13 @@
         <v>105</v>
       </c>
       <c r="H14" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="I14" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="J14" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="L14" s="4" t="s">
         <v>106</v>
@@ -2262,13 +2229,13 @@
         <v>109</v>
       </c>
       <c r="H15" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="I15" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="J15" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="L15" s="18" t="s">
         <v>110</v>
@@ -2302,13 +2269,13 @@
         <v>116</v>
       </c>
       <c r="H16" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="I16" s="8" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="J16" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="L16" s="4" t="s">
         <v>117</v>
@@ -2331,821 +2298,779 @@
         <v>120</v>
       </c>
       <c r="C17" t="s">
+        <v>120</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>122</v>
       </c>
-      <c r="E17" t="s">
-        <v>123</v>
-      </c>
       <c r="G17" s="4" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="H17" t="s">
-        <v>290</v>
-      </c>
-      <c r="I17" t="s">
-        <v>234</v>
+        <v>120</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>121</v>
       </c>
       <c r="J17" t="s">
-        <v>318</v>
+        <v>122</v>
       </c>
       <c r="L17" s="4" t="s">
-        <v>125</v>
+        <v>86</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="N17" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="O17" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="P17" s="4"/>
-      <c r="Q17" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="P17" s="7"/>
     </row>
     <row r="18" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C18" t="s">
+        <v>125</v>
+      </c>
+      <c r="D18" t="s">
+        <v>126</v>
+      </c>
+      <c r="E18" t="s">
         <v>127</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="C18" t="s">
-        <v>128</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="E18" t="s">
-        <v>130</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>128</v>
       </c>
       <c r="H18" t="s">
-        <v>128</v>
-      </c>
-      <c r="I18" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="I18" t="s">
+        <v>226</v>
+      </c>
+      <c r="J18" t="s">
+        <v>308</v>
+      </c>
+      <c r="L18" s="4" t="s">
         <v>129</v>
-      </c>
-      <c r="J18" t="s">
-        <v>130</v>
-      </c>
-      <c r="L18" s="4" t="s">
-        <v>86</v>
       </c>
       <c r="M18" s="4" t="s">
         <v>18</v>
       </c>
       <c r="N18" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="P18" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="P18" s="4"/>
     </row>
     <row r="19" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="C19" t="s">
         <v>132</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>133</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>134</v>
       </c>
-      <c r="E19" t="s">
+      <c r="G19" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="H19" t="s">
+        <v>282</v>
+      </c>
+      <c r="I19" t="s">
+        <v>227</v>
+      </c>
+      <c r="J19" t="s">
+        <v>309</v>
+      </c>
+      <c r="L19" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="M19" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="N19" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="O19" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="H19" t="s">
-        <v>291</v>
-      </c>
-      <c r="I19" t="s">
-        <v>235</v>
-      </c>
-      <c r="J19" t="s">
-        <v>319</v>
-      </c>
-      <c r="L19" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="M19" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N19" s="4" t="s">
-        <v>27</v>
-      </c>
       <c r="P19" s="4"/>
+      <c r="Q19" s="4"/>
     </row>
     <row r="20" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="C20" t="s">
+        <v>138</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E20" t="s">
+        <v>138</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="H20" t="s">
+        <v>283</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="J20" t="s">
+        <v>310</v>
+      </c>
+      <c r="L20" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="C20" t="s">
-        <v>140</v>
-      </c>
-      <c r="D20" t="s">
-        <v>141</v>
-      </c>
-      <c r="E20" t="s">
-        <v>142</v>
-      </c>
-      <c r="G20" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="H20" t="s">
-        <v>292</v>
-      </c>
-      <c r="I20" t="s">
-        <v>236</v>
-      </c>
-      <c r="J20" t="s">
-        <v>320</v>
-      </c>
-      <c r="L20" s="4" t="s">
-        <v>143</v>
-      </c>
       <c r="M20" s="4" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="N20" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="O20" s="4" t="s">
-        <v>144</v>
+        <v>19</v>
       </c>
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
     </row>
     <row r="21" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D21" t="s">
+        <v>143</v>
+      </c>
+      <c r="E21" t="s">
+        <v>144</v>
+      </c>
+      <c r="G21" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="H21" t="s">
+        <v>284</v>
+      </c>
+      <c r="I21" t="s">
+        <v>229</v>
+      </c>
+      <c r="J21" t="s">
+        <v>311</v>
+      </c>
+      <c r="L21" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="M21" s="4" t="s">
         <v>146</v>
-      </c>
-      <c r="C21" t="s">
-        <v>146</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E21" t="s">
-        <v>146</v>
-      </c>
-      <c r="G21" s="8" t="s">
-        <v>211</v>
-      </c>
-      <c r="H21" t="s">
-        <v>293</v>
-      </c>
-      <c r="I21" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="J21" t="s">
-        <v>321</v>
-      </c>
-      <c r="L21" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="M21" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="N21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="P21" s="4"/>
-      <c r="Q21" s="4"/>
     </row>
     <row r="22" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="D22" t="s">
-        <v>151</v>
-      </c>
-      <c r="E22" t="s">
-        <v>152</v>
-      </c>
-      <c r="G22" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="H22" t="s">
-        <v>294</v>
-      </c>
-      <c r="I22" t="s">
-        <v>238</v>
-      </c>
-      <c r="J22" t="s">
-        <v>322</v>
+      <c r="A22" s="19" t="s">
+        <v>349</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="E22" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="H22" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="I22" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="J22" s="18" t="s">
+        <v>348</v>
       </c>
       <c r="L22" s="18" t="s">
-        <v>153</v>
+        <v>110</v>
       </c>
       <c r="M22" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="N22" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="N22" s="18" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="19" t="s">
-        <v>360</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>355</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>355</v>
-      </c>
-      <c r="D23" s="18" t="s">
-        <v>355</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>355</v>
-      </c>
-      <c r="G23" s="18" t="s">
-        <v>356</v>
-      </c>
-      <c r="H23" s="18" t="s">
-        <v>357</v>
-      </c>
-      <c r="I23" s="18" t="s">
-        <v>358</v>
-      </c>
-      <c r="J23" s="18" t="s">
-        <v>359</v>
-      </c>
-      <c r="L23" s="18" t="s">
-        <v>110</v>
+      <c r="A23" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C23" t="s">
+        <v>149</v>
+      </c>
+      <c r="D23" t="s">
+        <v>150</v>
+      </c>
+      <c r="E23" t="s">
+        <v>151</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="H23" t="s">
+        <v>285</v>
+      </c>
+      <c r="I23" t="s">
+        <v>230</v>
+      </c>
+      <c r="J23" t="s">
+        <v>312</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>152</v>
       </c>
       <c r="M23" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="N23" s="4" t="s">
         <v>154</v>
-      </c>
-      <c r="N23" s="18" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="16" t="s">
+        <v>342</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>335</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>334</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="E24" s="15" t="s">
+        <v>336</v>
+      </c>
+      <c r="G24" s="15" t="s">
+        <v>337</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>338</v>
+      </c>
+      <c r="I24" s="15" t="s">
+        <v>339</v>
+      </c>
+      <c r="J24" s="15" t="s">
+        <v>340</v>
+      </c>
+      <c r="L24" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="M24" s="17" t="s">
+        <v>343</v>
+      </c>
+      <c r="N24" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C24" t="s">
-        <v>157</v>
-      </c>
-      <c r="D24" t="s">
-        <v>158</v>
-      </c>
-      <c r="E24" t="s">
-        <v>159</v>
-      </c>
-      <c r="G24" s="8" t="s">
-        <v>213</v>
-      </c>
-      <c r="H24" t="s">
-        <v>295</v>
-      </c>
-      <c r="I24" t="s">
-        <v>239</v>
-      </c>
-      <c r="J24" t="s">
-        <v>323</v>
-      </c>
-      <c r="L24" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="M24" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="N24" s="4" t="s">
-        <v>162</v>
-      </c>
+      <c r="P24" s="4"/>
+      <c r="Q24" s="4"/>
     </row>
     <row r="25" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="16" t="s">
-        <v>353</v>
-      </c>
-      <c r="B25" s="15" t="s">
-        <v>346</v>
-      </c>
-      <c r="C25" s="15" t="s">
-        <v>345</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>344</v>
-      </c>
-      <c r="E25" s="15" t="s">
-        <v>347</v>
-      </c>
-      <c r="G25" s="15" t="s">
-        <v>348</v>
-      </c>
-      <c r="H25" s="15" t="s">
-        <v>349</v>
-      </c>
-      <c r="I25" s="15" t="s">
-        <v>350</v>
-      </c>
-      <c r="J25" s="15" t="s">
-        <v>351</v>
+      <c r="A25" s="12" t="s">
+        <v>327</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="G25" s="13" t="s">
+        <v>328</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="I25" s="13" t="s">
+        <v>329</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>330</v>
       </c>
       <c r="L25" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="M25" s="17" t="s">
-        <v>354</v>
+        <v>155</v>
+      </c>
+      <c r="M25" s="13" t="s">
+        <v>170</v>
       </c>
       <c r="N25" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
     </row>
     <row r="26" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="12" t="s">
-        <v>338</v>
-      </c>
-      <c r="B26" s="13" t="s">
-        <v>339</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>342</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>340</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="G26" s="13" t="s">
-        <v>339</v>
-      </c>
-      <c r="H26" s="13" t="s">
-        <v>342</v>
-      </c>
-      <c r="I26" s="13" t="s">
-        <v>340</v>
-      </c>
-      <c r="J26" s="4" t="s">
-        <v>341</v>
+      <c r="A26" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="H26" t="s">
+        <v>286</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="J26" t="s">
+        <v>313</v>
       </c>
       <c r="L26" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="M26" s="13" t="s">
-        <v>178</v>
+        <v>158</v>
+      </c>
+      <c r="M26" s="4" t="s">
+        <v>159</v>
       </c>
       <c r="N26" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
     </row>
     <row r="27" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="D27" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="E27" s="8" t="s">
-        <v>256</v>
+      <c r="A27" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C27" t="s">
+        <v>161</v>
+      </c>
+      <c r="D27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E27" t="s">
+        <v>163</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>274</v>
+        <v>242</v>
       </c>
       <c r="H27" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="J27" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="L27" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="M27" s="4" t="s">
-        <v>167</v>
+        <v>164</v>
+      </c>
+      <c r="M27" s="17" t="s">
+        <v>343</v>
       </c>
       <c r="N27" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="P27" s="4"/>
-      <c r="Q27" s="4"/>
+        <v>156</v>
+      </c>
     </row>
     <row r="28" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="16" t="s">
-        <v>352</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="C28" t="s">
-        <v>169</v>
-      </c>
-      <c r="D28" t="s">
-        <v>170</v>
-      </c>
-      <c r="E28" t="s">
-        <v>171</v>
+      <c r="A28" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>260</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>251</v>
+        <v>206</v>
       </c>
       <c r="H28" t="s">
-        <v>297</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>275</v>
+        <v>288</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>231</v>
       </c>
       <c r="J28" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="L28" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="M28" s="17" t="s">
-        <v>354</v>
+        <v>166</v>
+      </c>
+      <c r="M28" s="4" t="s">
+        <v>167</v>
       </c>
       <c r="N28" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="29" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="3" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="H29" t="s">
-        <v>298</v>
+        <v>207</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>289</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="J29" t="s">
-        <v>326</v>
+        <v>232</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>316</v>
       </c>
       <c r="L29" s="4" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="M29" s="4" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="N29" s="4" t="s">
-        <v>164</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="P29" s="4"/>
+      <c r="Q29" s="4"/>
     </row>
     <row r="30" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>253</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>258</v>
+        <v>171</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="C30" t="s">
+        <v>173</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>262</v>
-      </c>
-      <c r="E30" s="8" t="s">
-        <v>273</v>
+        <v>174</v>
+      </c>
+      <c r="E30" t="s">
+        <v>175</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>215</v>
-      </c>
-      <c r="H30" s="4" t="s">
-        <v>299</v>
-      </c>
-      <c r="I30" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="J30" s="4" t="s">
-        <v>327</v>
+        <v>213</v>
+      </c>
+      <c r="H30" t="s">
+        <v>290</v>
+      </c>
+      <c r="I30" t="s">
+        <v>233</v>
+      </c>
+      <c r="J30" t="s">
+        <v>317</v>
       </c>
       <c r="L30" s="4" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="M30" s="4" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="N30" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="P30" s="4"/>
-      <c r="Q30" s="4"/>
+        <v>156</v>
+      </c>
     </row>
     <row r="31" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C31" t="s">
+        <v>178</v>
+      </c>
+      <c r="D31" t="s">
         <v>179</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="E31" t="s">
         <v>180</v>
       </c>
-      <c r="C31" t="s">
-        <v>181</v>
-      </c>
-      <c r="D31" s="8" t="s">
-        <v>182</v>
-      </c>
-      <c r="E31" t="s">
-        <v>183</v>
-      </c>
       <c r="G31" s="8" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="H31" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="I31" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="J31" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="L31" s="4" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="M31" s="4" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="N31" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="C32" t="s">
-        <v>186</v>
-      </c>
-      <c r="D32" t="s">
-        <v>187</v>
-      </c>
-      <c r="E32" t="s">
-        <v>188</v>
+        <v>181</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>261</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="H32" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="I32" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="J32" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="L32" s="4" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="M32" s="4" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="N32" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="33" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="3" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="H33" t="s">
-        <v>302</v>
-      </c>
-      <c r="I33" t="s">
-        <v>244</v>
-      </c>
-      <c r="J33" t="s">
-        <v>330</v>
+        <v>209</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="I33" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>320</v>
       </c>
       <c r="L33" s="4" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="M33" s="4" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="N33" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="C34" t="s">
+        <v>189</v>
+      </c>
+      <c r="D34" t="s">
+        <v>190</v>
+      </c>
+      <c r="E34" t="s">
+        <v>191</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="H34" t="s">
+        <v>294</v>
+      </c>
+      <c r="I34" t="s">
+        <v>237</v>
+      </c>
+      <c r="J34" t="s">
+        <v>321</v>
+      </c>
+      <c r="L34" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>265</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="D34" s="8" t="s">
-        <v>266</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>271</v>
-      </c>
-      <c r="G34" s="8" t="s">
-        <v>217</v>
-      </c>
-      <c r="H34" s="4" t="s">
-        <v>303</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="J34" s="4" t="s">
-        <v>331</v>
-      </c>
-      <c r="L34" s="4" t="s">
+      <c r="M34" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="M34" s="4" t="s">
-        <v>194</v>
-      </c>
       <c r="N34" s="4" t="s">
-        <v>164</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="P34" s="4"/>
     </row>
     <row r="35" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="H35" t="s">
+        <v>295</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="J35" t="s">
+        <v>322</v>
+      </c>
+      <c r="L35" s="4" t="s">
         <v>195</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="M35" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="C35" t="s">
-        <v>197</v>
-      </c>
-      <c r="D35" t="s">
-        <v>198</v>
-      </c>
-      <c r="E35" t="s">
-        <v>199</v>
-      </c>
-      <c r="G35" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="H35" t="s">
-        <v>304</v>
-      </c>
-      <c r="I35" t="s">
-        <v>246</v>
-      </c>
-      <c r="J35" t="s">
-        <v>332</v>
-      </c>
-      <c r="L35" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="M35" s="4" t="s">
-        <v>201</v>
-      </c>
       <c r="N35" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="P35" s="4"/>
+      <c r="Q35" s="4"/>
     </row>
     <row r="36" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D36" s="8" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H36" t="s">
-        <v>305</v>
-      </c>
-      <c r="I36" s="4" t="s">
-        <v>247</v>
+        <v>296</v>
+      </c>
+      <c r="I36" t="s">
+        <v>239</v>
       </c>
       <c r="J36" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
       <c r="L36" s="4" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="M36" s="4" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="N36" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="P36" s="4"/>
-      <c r="Q36" s="4"/>
+        <v>156</v>
+      </c>
     </row>
-    <row r="37" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B37" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>261</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>268</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>272</v>
-      </c>
-      <c r="G37" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="H37" t="s">
-        <v>306</v>
-      </c>
-      <c r="I37" t="s">
-        <v>248</v>
-      </c>
-      <c r="J37" t="s">
-        <v>334</v>
-      </c>
-      <c r="L37" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="M37" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="N37" s="4" t="s">
-        <v>164</v>
-      </c>
-    </row>
+    <row r="37" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="38" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="39" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="40" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4020,9 +3945,8 @@
     <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <autoFilter ref="A1:Q37" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:Q36" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="A1" r:id="rId1" location="property-name" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B1" r:id="rId2" location="property-labels" xr:uid="{00000000-0004-0000-0000-000001000000}"/>

</xml_diff>